<commit_message>
fix: import export ticket paymentDate
</commit_message>
<xml_diff>
--- a/__fixtures__/simple-lcra.xlsx
+++ b/__fixtures__/simple-lcra.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11028"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D2FD1F-9472-BF42-9EC0-D4AE4C9794A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kendrick/Documents/git/community-db/__fixtures__/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB636ACE-3629-4846-A35B-929441705A7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="65880" yWindow="-600" windowWidth="33940" windowHeight="26860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1520" yWindow="600" windowWidth="49680" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sample Community" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="95">
   <si>
     <t>Address</t>
   </si>
@@ -29,21 +34,27 @@
     <t>PostalCode</t>
   </si>
   <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>LastModDate</t>
+  </si>
+  <si>
+    <t>LastModBy</t>
+  </si>
+  <si>
     <t>FirstName1</t>
   </si>
   <si>
     <t>LastName1</t>
   </si>
   <si>
+    <t>EMail1OptOut</t>
+  </si>
+  <si>
     <t>EMail1</t>
   </si>
   <si>
-    <t>EMail1Facebook</t>
-  </si>
-  <si>
-    <t>EMail1OptOut</t>
-  </si>
-  <si>
     <t>HomePhone1</t>
   </si>
   <si>
@@ -59,15 +70,12 @@
     <t>LastName2</t>
   </si>
   <si>
+    <t>EMail2OptOut</t>
+  </si>
+  <si>
     <t>EMail2</t>
   </si>
   <si>
-    <t>EMail2Facebook</t>
-  </si>
-  <si>
-    <t>EMail2OptOut</t>
-  </si>
-  <si>
     <t>HomePhone2</t>
   </si>
   <si>
@@ -83,15 +91,12 @@
     <t>LastName3</t>
   </si>
   <si>
+    <t>EMail3OptOut</t>
+  </si>
+  <si>
     <t>EMail3</t>
   </si>
   <si>
-    <t>EMail3Facebook</t>
-  </si>
-  <si>
-    <t>EMail3OptOut</t>
-  </si>
-  <si>
     <t>HomePhone3</t>
   </si>
   <si>
@@ -101,39 +106,6 @@
     <t>CellPhone3</t>
   </si>
   <si>
-    <t>FirstName4</t>
-  </si>
-  <si>
-    <t>LastName4</t>
-  </si>
-  <si>
-    <t>EMail4</t>
-  </si>
-  <si>
-    <t>EMail4Facebook</t>
-  </si>
-  <si>
-    <t>EMail4OptOut</t>
-  </si>
-  <si>
-    <t>HomePhone4</t>
-  </si>
-  <si>
-    <t>WorkPhone4</t>
-  </si>
-  <si>
-    <t>CellPhone4</t>
-  </si>
-  <si>
-    <t>LastModDate</t>
-  </si>
-  <si>
-    <t>LastModBy</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
     <t>Y24</t>
   </si>
   <si>
@@ -143,12 +115,18 @@
     <t>Y24-date</t>
   </si>
   <si>
+    <t>Y24-ticket</t>
+  </si>
+  <si>
     <t>Y24-payment</t>
   </si>
   <si>
     <t>Y24-deposited</t>
   </si>
   <si>
+    <t>Y24-price</t>
+  </si>
+  <si>
     <t>Y23</t>
   </si>
   <si>
@@ -158,12 +136,18 @@
     <t>Y23-date</t>
   </si>
   <si>
+    <t>Y23-ticket</t>
+  </si>
+  <si>
     <t>Y23-payment</t>
   </si>
   <si>
     <t>Y23-deposited</t>
   </si>
   <si>
+    <t>Y23-price</t>
+  </si>
+  <si>
     <t>Y22</t>
   </si>
   <si>
@@ -173,12 +157,18 @@
     <t>Y22-date</t>
   </si>
   <si>
+    <t>Y22-ticket</t>
+  </si>
+  <si>
     <t>Y22-payment</t>
   </si>
   <si>
     <t>Y22-deposited</t>
   </si>
   <si>
+    <t>Y22-price</t>
+  </si>
+  <si>
     <t>Y21</t>
   </si>
   <si>
@@ -188,133 +178,143 @@
     <t>Y21-date</t>
   </si>
   <si>
+    <t>Y21-ticket</t>
+  </si>
+  <si>
     <t>Y21-payment</t>
   </si>
   <si>
     <t>Y21-deposited</t>
   </si>
   <si>
+    <t>Y21-price</t>
+  </si>
+  <si>
+    <t>123 Adventure Drive</t>
+  </si>
+  <si>
+    <t>Adventure Drive</t>
+  </si>
+  <si>
+    <t>A0A0A0</t>
+  </si>
+  <si>
+    <t>2nd entry</t>
+  </si>
+  <si>
+    <t>2023-02-23T03:19:09.000Z</t>
+  </si>
+  <si>
+    <t>test@email.com</t>
+  </si>
+  <si>
+    <t>Kevin</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>ksmith@email.com</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>2023-02-23T03:19:09+00:00</t>
+    <t>Corn Roast</t>
+  </si>
+  <si>
+    <t>2023-08-20T00:00:00.000Z</t>
+  </si>
+  <si>
+    <t>meal:20:0:free:/drink:1:1:cash:2023-08-21T000000.000Z</t>
+  </si>
+  <si>
+    <t>cash</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>99 Fortune Drive</t>
+  </si>
+  <si>
+    <t>Fortune Drive</t>
+  </si>
+  <si>
+    <t>First1</t>
+  </si>
+  <si>
+    <t>Last1</t>
+  </si>
+  <si>
+    <t>Email1</t>
+  </si>
+  <si>
+    <t>4161234567</t>
+  </si>
+  <si>
+    <t>4162345678</t>
+  </si>
+  <si>
+    <t>4163456789</t>
+  </si>
+  <si>
+    <t>First2</t>
+  </si>
+  <si>
+    <t>Last2</t>
+  </si>
+  <si>
+    <t>Email2</t>
+  </si>
+  <si>
+    <t>4171234567</t>
+  </si>
+  <si>
+    <t>First3</t>
+  </si>
+  <si>
+    <t>Last3</t>
+  </si>
+  <si>
+    <t>Email3</t>
+  </si>
+  <si>
+    <t>Summer Festival;Corn Roast</t>
+  </si>
+  <si>
+    <t>2023-06-11T00:00:00.000Z;2023-08-20T00:00:00.000Z</t>
+  </si>
+  <si>
+    <t>meal:20:0:free:/cotton-candy:1:1:cash:2023-06-12T000000.000Z;meal:10:5:cash:/drink:1:1:e-Transfer:</t>
   </si>
   <si>
     <t>e-Transfer</t>
   </si>
   <si>
+    <t>10</t>
+  </si>
+  <si>
     <t>Membership Carry Forward</t>
   </si>
   <si>
-    <t>2022-02-10T20:34:21-05:00</t>
+    <t>2022-02-10T00:00:00.000Z</t>
   </si>
   <si>
     <t>free</t>
   </si>
   <si>
-    <t>2021-01-23T22:27:40-05:00</t>
-  </si>
-  <si>
-    <t>99 Fortune Drive</t>
-  </si>
-  <si>
-    <t>Fortune Drive</t>
-  </si>
-  <si>
-    <t>A0A0A0</t>
-  </si>
-  <si>
-    <t>First1</t>
-  </si>
-  <si>
-    <t>First2</t>
-  </si>
-  <si>
-    <t>Email1</t>
-  </si>
-  <si>
-    <t>Last2</t>
-  </si>
-  <si>
-    <t>Email2</t>
-  </si>
-  <si>
-    <t>First3</t>
-  </si>
-  <si>
-    <t>Last3</t>
-  </si>
-  <si>
-    <t>Email3</t>
-  </si>
-  <si>
-    <t>Last1</t>
-  </si>
-  <si>
-    <t>Summer Festival;Corn Roast</t>
-  </si>
-  <si>
-    <t>2023-06-11T16:00:00-04:00;2023-08-20T17:07:25-04:00</t>
-  </si>
-  <si>
-    <t>123 Adventure Drive</t>
-  </si>
-  <si>
-    <t>Adventure Drive</t>
-  </si>
-  <si>
-    <t>Kevin</t>
-  </si>
-  <si>
-    <t>Smith</t>
-  </si>
-  <si>
-    <t>ksmith@email.com</t>
-  </si>
-  <si>
-    <t>2nd entry</t>
-  </si>
-  <si>
-    <t>Corn Roast</t>
-  </si>
-  <si>
-    <t>cash</t>
-  </si>
-  <si>
-    <t>2023-08-20T17:07:25-04:00</t>
-  </si>
-  <si>
-    <t>test@email.com</t>
-  </si>
-  <si>
-    <t>Y23-ticket</t>
-  </si>
-  <si>
-    <t>meal:20:0:free/drink:1:1:cash</t>
-  </si>
-  <si>
-    <t>Y23-price</t>
-  </si>
-  <si>
-    <t>meal:20:0:free/cotton-candy:1:1:cash;meal:10:5:cash/drink:1:1:e-Transfer</t>
+    <t>2021-01-23T00:00:00.000Z</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -337,20 +337,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -684,29 +681,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BI3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="4" max="4" width="11.5" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="9" max="9" width="15.33203125" customWidth="1"/>
-    <col min="10" max="12" width="12" customWidth="1"/>
-    <col min="18" max="20" width="12" customWidth="1"/>
-    <col min="26" max="28" width="12" customWidth="1"/>
-    <col min="34" max="36" width="12" customWidth="1"/>
-    <col min="37" max="37" width="19.6640625" customWidth="1"/>
-    <col min="38" max="38" width="16" customWidth="1"/>
-    <col min="39" max="39" width="40" customWidth="1"/>
-    <col min="44" max="44" width="24.83203125" customWidth="1"/>
-    <col min="46" max="46" width="27.6640625" customWidth="1"/>
-    <col min="47" max="47" width="47" customWidth="1"/>
-    <col min="48" max="48" width="11.1640625" customWidth="1"/>
-    <col min="51" max="51" width="72.5" customWidth="1"/>
-    <col min="59" max="59" width="16" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:BD3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -849,274 +827,272 @@
         <v>46</v>
       </c>
       <c r="AV1" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="AW1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="AX1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="AY1" t="s">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="AZ1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="BA1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="BB1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="BC1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="BD1" t="s">
-        <v>53</v>
-      </c>
-      <c r="BE1" t="s">
-        <v>54</v>
-      </c>
-      <c r="BF1" t="s">
         <v>55</v>
       </c>
-      <c r="BG1" t="s">
+    </row>
+    <row r="2" spans="1:56" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>56</v>
-      </c>
-      <c r="BH1" t="s">
-        <v>57</v>
-      </c>
-      <c r="BI1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="2" spans="1:61" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>80</v>
       </c>
       <c r="B2">
         <v>123</v>
       </c>
       <c r="C2" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="D2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I2" t="s">
+        <v>63</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2" t="s">
+        <v>64</v>
+      </c>
+      <c r="AC2">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH2">
+        <v>0</v>
+      </c>
+      <c r="AJ2">
+        <v>1</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>66</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM2" t="s">
         <v>68</v>
       </c>
-      <c r="E2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F2" t="s">
-        <v>83</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL2" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AN2">
-        <v>0</v>
-      </c>
-      <c r="AO2" t="s">
-        <v>59</v>
+      <c r="AN2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AO2">
+        <v>1</v>
       </c>
       <c r="AP2" t="s">
-        <v>59</v>
-      </c>
-      <c r="AQ2" t="s">
-        <v>59</v>
-      </c>
-      <c r="AR2">
-        <v>0</v>
-      </c>
-      <c r="AS2">
-        <v>1</v>
+        <v>70</v>
+      </c>
+      <c r="AQ2">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AS2" t="s">
+        <v>65</v>
       </c>
       <c r="AT2" t="s">
-        <v>86</v>
-      </c>
-      <c r="AU2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AV2">
-        <v>20</v>
-      </c>
-      <c r="AW2" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="AX2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AZ2">
-        <v>0</v>
-      </c>
-      <c r="BE2">
-        <v>0</v>
-      </c>
-      <c r="BI2">
+        <v>65</v>
+      </c>
+      <c r="AZ2" t="s">
+        <v>65</v>
+      </c>
+      <c r="BA2" t="s">
+        <v>65</v>
+      </c>
+      <c r="BC2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B3">
         <v>99</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D3" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="E3" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="F3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" t="s">
+        <v>73</v>
+      </c>
+      <c r="I3" t="s">
+        <v>74</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3" t="s">
+        <v>75</v>
+      </c>
+      <c r="L3" t="s">
+        <v>76</v>
+      </c>
+      <c r="M3" t="s">
         <v>77</v>
       </c>
-      <c r="G3" t="s">
-        <v>71</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
-        <v>4161234567</v>
-      </c>
-      <c r="K3">
-        <v>4162345678</v>
-      </c>
-      <c r="L3">
-        <v>4163456789</v>
-      </c>
-      <c r="M3" t="s">
-        <v>70</v>
-      </c>
       <c r="N3" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="O3" t="s">
-        <v>73</v>
-      </c>
-      <c r="P3">
-        <v>0</v>
+        <v>79</v>
+      </c>
+      <c r="P3" t="s">
+        <v>80</v>
       </c>
       <c r="Q3">
         <v>1</v>
       </c>
-      <c r="R3">
-        <v>4171234567</v>
-      </c>
-      <c r="U3" t="s">
-        <v>74</v>
+      <c r="R3" t="s">
+        <v>81</v>
+      </c>
+      <c r="S3" t="s">
+        <v>82</v>
       </c>
       <c r="V3" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="W3" t="s">
-        <v>76</v>
+        <v>84</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>85</v>
+      </c>
+      <c r="AC3">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH3">
+        <v>0</v>
+      </c>
+      <c r="AJ3">
+        <v>1</v>
       </c>
       <c r="AK3" t="s">
-        <v>60</v>
+        <v>86</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>87</v>
       </c>
       <c r="AM3" t="s">
-        <v>38</v>
-      </c>
-      <c r="AN3">
-        <v>0</v>
-      </c>
-      <c r="AO3" t="s">
-        <v>59</v>
+        <v>88</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>89</v>
+      </c>
+      <c r="AO3">
+        <v>1</v>
       </c>
       <c r="AP3" t="s">
-        <v>59</v>
-      </c>
-      <c r="AQ3" t="s">
-        <v>59</v>
-      </c>
-      <c r="AR3">
-        <v>0</v>
-      </c>
-      <c r="AS3">
+        <v>90</v>
+      </c>
+      <c r="AQ3">
         <v>1</v>
       </c>
+      <c r="AR3" t="s">
+        <v>91</v>
+      </c>
+      <c r="AS3" t="s">
+        <v>92</v>
+      </c>
       <c r="AT3" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="AU3" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="AV3">
-        <v>10</v>
-      </c>
-      <c r="AW3" t="s">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="AX3">
         <v>1</v>
       </c>
       <c r="AY3" t="s">
+        <v>91</v>
+      </c>
+      <c r="AZ3" t="s">
+        <v>94</v>
+      </c>
+      <c r="BA3" t="s">
+        <v>65</v>
+      </c>
+      <c r="BB3" t="s">
         <v>93</v>
       </c>
-      <c r="AZ3">
-        <v>1</v>
-      </c>
-      <c r="BA3" t="s">
-        <v>62</v>
-      </c>
-      <c r="BB3" t="s">
-        <v>63</v>
-      </c>
-      <c r="BC3" t="s">
-        <v>64</v>
-      </c>
-      <c r="BD3">
-        <v>0</v>
-      </c>
-      <c r="BE3">
-        <v>1</v>
-      </c>
-      <c r="BF3" t="s">
-        <v>62</v>
-      </c>
-      <c r="BG3" t="s">
-        <v>65</v>
-      </c>
-      <c r="BH3" t="s">
-        <v>64</v>
-      </c>
-      <c r="BI3">
+      <c r="BC3">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{6B4B139F-5BD3-0642-96FD-B1E293BB7330}"/>
-    <hyperlink ref="AL2" r:id="rId2" xr:uid="{CD755D91-AB99-E442-AEBE-30FEAB99775E}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:BD3" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: reposition add ticket/add event button (#320)
</commit_message>
<xml_diff>
--- a/__fixtures__/simple-lcra.xlsx
+++ b/__fixtures__/simple-lcra.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11028"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D2FD1F-9472-BF42-9EC0-D4AE4C9794A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kendrick/Documents/git/community-db/__fixtures__/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB636ACE-3629-4846-A35B-929441705A7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="65880" yWindow="-600" windowWidth="33940" windowHeight="26860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1520" yWindow="600" windowWidth="49680" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sample Community" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="95">
   <si>
     <t>Address</t>
   </si>
@@ -29,21 +34,27 @@
     <t>PostalCode</t>
   </si>
   <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>LastModDate</t>
+  </si>
+  <si>
+    <t>LastModBy</t>
+  </si>
+  <si>
     <t>FirstName1</t>
   </si>
   <si>
     <t>LastName1</t>
   </si>
   <si>
+    <t>EMail1OptOut</t>
+  </si>
+  <si>
     <t>EMail1</t>
   </si>
   <si>
-    <t>EMail1Facebook</t>
-  </si>
-  <si>
-    <t>EMail1OptOut</t>
-  </si>
-  <si>
     <t>HomePhone1</t>
   </si>
   <si>
@@ -59,15 +70,12 @@
     <t>LastName2</t>
   </si>
   <si>
+    <t>EMail2OptOut</t>
+  </si>
+  <si>
     <t>EMail2</t>
   </si>
   <si>
-    <t>EMail2Facebook</t>
-  </si>
-  <si>
-    <t>EMail2OptOut</t>
-  </si>
-  <si>
     <t>HomePhone2</t>
   </si>
   <si>
@@ -83,15 +91,12 @@
     <t>LastName3</t>
   </si>
   <si>
+    <t>EMail3OptOut</t>
+  </si>
+  <si>
     <t>EMail3</t>
   </si>
   <si>
-    <t>EMail3Facebook</t>
-  </si>
-  <si>
-    <t>EMail3OptOut</t>
-  </si>
-  <si>
     <t>HomePhone3</t>
   </si>
   <si>
@@ -101,39 +106,6 @@
     <t>CellPhone3</t>
   </si>
   <si>
-    <t>FirstName4</t>
-  </si>
-  <si>
-    <t>LastName4</t>
-  </si>
-  <si>
-    <t>EMail4</t>
-  </si>
-  <si>
-    <t>EMail4Facebook</t>
-  </si>
-  <si>
-    <t>EMail4OptOut</t>
-  </si>
-  <si>
-    <t>HomePhone4</t>
-  </si>
-  <si>
-    <t>WorkPhone4</t>
-  </si>
-  <si>
-    <t>CellPhone4</t>
-  </si>
-  <si>
-    <t>LastModDate</t>
-  </si>
-  <si>
-    <t>LastModBy</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
     <t>Y24</t>
   </si>
   <si>
@@ -143,12 +115,18 @@
     <t>Y24-date</t>
   </si>
   <si>
+    <t>Y24-ticket</t>
+  </si>
+  <si>
     <t>Y24-payment</t>
   </si>
   <si>
     <t>Y24-deposited</t>
   </si>
   <si>
+    <t>Y24-price</t>
+  </si>
+  <si>
     <t>Y23</t>
   </si>
   <si>
@@ -158,12 +136,18 @@
     <t>Y23-date</t>
   </si>
   <si>
+    <t>Y23-ticket</t>
+  </si>
+  <si>
     <t>Y23-payment</t>
   </si>
   <si>
     <t>Y23-deposited</t>
   </si>
   <si>
+    <t>Y23-price</t>
+  </si>
+  <si>
     <t>Y22</t>
   </si>
   <si>
@@ -173,12 +157,18 @@
     <t>Y22-date</t>
   </si>
   <si>
+    <t>Y22-ticket</t>
+  </si>
+  <si>
     <t>Y22-payment</t>
   </si>
   <si>
     <t>Y22-deposited</t>
   </si>
   <si>
+    <t>Y22-price</t>
+  </si>
+  <si>
     <t>Y21</t>
   </si>
   <si>
@@ -188,133 +178,143 @@
     <t>Y21-date</t>
   </si>
   <si>
+    <t>Y21-ticket</t>
+  </si>
+  <si>
     <t>Y21-payment</t>
   </si>
   <si>
     <t>Y21-deposited</t>
   </si>
   <si>
+    <t>Y21-price</t>
+  </si>
+  <si>
+    <t>123 Adventure Drive</t>
+  </si>
+  <si>
+    <t>Adventure Drive</t>
+  </si>
+  <si>
+    <t>A0A0A0</t>
+  </si>
+  <si>
+    <t>2nd entry</t>
+  </si>
+  <si>
+    <t>2023-02-23T03:19:09.000Z</t>
+  </si>
+  <si>
+    <t>test@email.com</t>
+  </si>
+  <si>
+    <t>Kevin</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>ksmith@email.com</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>2023-02-23T03:19:09+00:00</t>
+    <t>Corn Roast</t>
+  </si>
+  <si>
+    <t>2023-08-20T00:00:00.000Z</t>
+  </si>
+  <si>
+    <t>meal:20:0:free:/drink:1:1:cash:2023-08-21T000000.000Z</t>
+  </si>
+  <si>
+    <t>cash</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>99 Fortune Drive</t>
+  </si>
+  <si>
+    <t>Fortune Drive</t>
+  </si>
+  <si>
+    <t>First1</t>
+  </si>
+  <si>
+    <t>Last1</t>
+  </si>
+  <si>
+    <t>Email1</t>
+  </si>
+  <si>
+    <t>4161234567</t>
+  </si>
+  <si>
+    <t>4162345678</t>
+  </si>
+  <si>
+    <t>4163456789</t>
+  </si>
+  <si>
+    <t>First2</t>
+  </si>
+  <si>
+    <t>Last2</t>
+  </si>
+  <si>
+    <t>Email2</t>
+  </si>
+  <si>
+    <t>4171234567</t>
+  </si>
+  <si>
+    <t>First3</t>
+  </si>
+  <si>
+    <t>Last3</t>
+  </si>
+  <si>
+    <t>Email3</t>
+  </si>
+  <si>
+    <t>Summer Festival;Corn Roast</t>
+  </si>
+  <si>
+    <t>2023-06-11T00:00:00.000Z;2023-08-20T00:00:00.000Z</t>
+  </si>
+  <si>
+    <t>meal:20:0:free:/cotton-candy:1:1:cash:2023-06-12T000000.000Z;meal:10:5:cash:/drink:1:1:e-Transfer:</t>
   </si>
   <si>
     <t>e-Transfer</t>
   </si>
   <si>
+    <t>10</t>
+  </si>
+  <si>
     <t>Membership Carry Forward</t>
   </si>
   <si>
-    <t>2022-02-10T20:34:21-05:00</t>
+    <t>2022-02-10T00:00:00.000Z</t>
   </si>
   <si>
     <t>free</t>
   </si>
   <si>
-    <t>2021-01-23T22:27:40-05:00</t>
-  </si>
-  <si>
-    <t>99 Fortune Drive</t>
-  </si>
-  <si>
-    <t>Fortune Drive</t>
-  </si>
-  <si>
-    <t>A0A0A0</t>
-  </si>
-  <si>
-    <t>First1</t>
-  </si>
-  <si>
-    <t>First2</t>
-  </si>
-  <si>
-    <t>Email1</t>
-  </si>
-  <si>
-    <t>Last2</t>
-  </si>
-  <si>
-    <t>Email2</t>
-  </si>
-  <si>
-    <t>First3</t>
-  </si>
-  <si>
-    <t>Last3</t>
-  </si>
-  <si>
-    <t>Email3</t>
-  </si>
-  <si>
-    <t>Last1</t>
-  </si>
-  <si>
-    <t>Summer Festival;Corn Roast</t>
-  </si>
-  <si>
-    <t>2023-06-11T16:00:00-04:00;2023-08-20T17:07:25-04:00</t>
-  </si>
-  <si>
-    <t>123 Adventure Drive</t>
-  </si>
-  <si>
-    <t>Adventure Drive</t>
-  </si>
-  <si>
-    <t>Kevin</t>
-  </si>
-  <si>
-    <t>Smith</t>
-  </si>
-  <si>
-    <t>ksmith@email.com</t>
-  </si>
-  <si>
-    <t>2nd entry</t>
-  </si>
-  <si>
-    <t>Corn Roast</t>
-  </si>
-  <si>
-    <t>cash</t>
-  </si>
-  <si>
-    <t>2023-08-20T17:07:25-04:00</t>
-  </si>
-  <si>
-    <t>test@email.com</t>
-  </si>
-  <si>
-    <t>Y23-ticket</t>
-  </si>
-  <si>
-    <t>meal:20:0:free/drink:1:1:cash</t>
-  </si>
-  <si>
-    <t>Y23-price</t>
-  </si>
-  <si>
-    <t>meal:20:0:free/cotton-candy:1:1:cash;meal:10:5:cash/drink:1:1:e-Transfer</t>
+    <t>2021-01-23T00:00:00.000Z</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -337,20 +337,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -684,29 +681,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BI3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="4" max="4" width="11.5" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="9" max="9" width="15.33203125" customWidth="1"/>
-    <col min="10" max="12" width="12" customWidth="1"/>
-    <col min="18" max="20" width="12" customWidth="1"/>
-    <col min="26" max="28" width="12" customWidth="1"/>
-    <col min="34" max="36" width="12" customWidth="1"/>
-    <col min="37" max="37" width="19.6640625" customWidth="1"/>
-    <col min="38" max="38" width="16" customWidth="1"/>
-    <col min="39" max="39" width="40" customWidth="1"/>
-    <col min="44" max="44" width="24.83203125" customWidth="1"/>
-    <col min="46" max="46" width="27.6640625" customWidth="1"/>
-    <col min="47" max="47" width="47" customWidth="1"/>
-    <col min="48" max="48" width="11.1640625" customWidth="1"/>
-    <col min="51" max="51" width="72.5" customWidth="1"/>
-    <col min="59" max="59" width="16" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:BD3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -849,274 +827,272 @@
         <v>46</v>
       </c>
       <c r="AV1" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="AW1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="AX1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="AY1" t="s">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="AZ1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="BA1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="BB1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="BC1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="BD1" t="s">
-        <v>53</v>
-      </c>
-      <c r="BE1" t="s">
-        <v>54</v>
-      </c>
-      <c r="BF1" t="s">
         <v>55</v>
       </c>
-      <c r="BG1" t="s">
+    </row>
+    <row r="2" spans="1:56" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>56</v>
-      </c>
-      <c r="BH1" t="s">
-        <v>57</v>
-      </c>
-      <c r="BI1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="2" spans="1:61" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>80</v>
       </c>
       <c r="B2">
         <v>123</v>
       </c>
       <c r="C2" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="D2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I2" t="s">
+        <v>63</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2" t="s">
+        <v>64</v>
+      </c>
+      <c r="AC2">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH2">
+        <v>0</v>
+      </c>
+      <c r="AJ2">
+        <v>1</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>66</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM2" t="s">
         <v>68</v>
       </c>
-      <c r="E2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F2" t="s">
-        <v>83</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL2" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AN2">
-        <v>0</v>
-      </c>
-      <c r="AO2" t="s">
-        <v>59</v>
+      <c r="AN2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AO2">
+        <v>1</v>
       </c>
       <c r="AP2" t="s">
-        <v>59</v>
-      </c>
-      <c r="AQ2" t="s">
-        <v>59</v>
-      </c>
-      <c r="AR2">
-        <v>0</v>
-      </c>
-      <c r="AS2">
-        <v>1</v>
+        <v>70</v>
+      </c>
+      <c r="AQ2">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AS2" t="s">
+        <v>65</v>
       </c>
       <c r="AT2" t="s">
-        <v>86</v>
-      </c>
-      <c r="AU2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AV2">
-        <v>20</v>
-      </c>
-      <c r="AW2" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="AX2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AZ2">
-        <v>0</v>
-      </c>
-      <c r="BE2">
-        <v>0</v>
-      </c>
-      <c r="BI2">
+        <v>65</v>
+      </c>
+      <c r="AZ2" t="s">
+        <v>65</v>
+      </c>
+      <c r="BA2" t="s">
+        <v>65</v>
+      </c>
+      <c r="BC2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B3">
         <v>99</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D3" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="E3" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="F3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" t="s">
+        <v>73</v>
+      </c>
+      <c r="I3" t="s">
+        <v>74</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3" t="s">
+        <v>75</v>
+      </c>
+      <c r="L3" t="s">
+        <v>76</v>
+      </c>
+      <c r="M3" t="s">
         <v>77</v>
       </c>
-      <c r="G3" t="s">
-        <v>71</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
-        <v>4161234567</v>
-      </c>
-      <c r="K3">
-        <v>4162345678</v>
-      </c>
-      <c r="L3">
-        <v>4163456789</v>
-      </c>
-      <c r="M3" t="s">
-        <v>70</v>
-      </c>
       <c r="N3" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="O3" t="s">
-        <v>73</v>
-      </c>
-      <c r="P3">
-        <v>0</v>
+        <v>79</v>
+      </c>
+      <c r="P3" t="s">
+        <v>80</v>
       </c>
       <c r="Q3">
         <v>1</v>
       </c>
-      <c r="R3">
-        <v>4171234567</v>
-      </c>
-      <c r="U3" t="s">
-        <v>74</v>
+      <c r="R3" t="s">
+        <v>81</v>
+      </c>
+      <c r="S3" t="s">
+        <v>82</v>
       </c>
       <c r="V3" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="W3" t="s">
-        <v>76</v>
+        <v>84</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>85</v>
+      </c>
+      <c r="AC3">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH3">
+        <v>0</v>
+      </c>
+      <c r="AJ3">
+        <v>1</v>
       </c>
       <c r="AK3" t="s">
-        <v>60</v>
+        <v>86</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>87</v>
       </c>
       <c r="AM3" t="s">
-        <v>38</v>
-      </c>
-      <c r="AN3">
-        <v>0</v>
-      </c>
-      <c r="AO3" t="s">
-        <v>59</v>
+        <v>88</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>89</v>
+      </c>
+      <c r="AO3">
+        <v>1</v>
       </c>
       <c r="AP3" t="s">
-        <v>59</v>
-      </c>
-      <c r="AQ3" t="s">
-        <v>59</v>
-      </c>
-      <c r="AR3">
-        <v>0</v>
-      </c>
-      <c r="AS3">
+        <v>90</v>
+      </c>
+      <c r="AQ3">
         <v>1</v>
       </c>
+      <c r="AR3" t="s">
+        <v>91</v>
+      </c>
+      <c r="AS3" t="s">
+        <v>92</v>
+      </c>
       <c r="AT3" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="AU3" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="AV3">
-        <v>10</v>
-      </c>
-      <c r="AW3" t="s">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="AX3">
         <v>1</v>
       </c>
       <c r="AY3" t="s">
+        <v>91</v>
+      </c>
+      <c r="AZ3" t="s">
+        <v>94</v>
+      </c>
+      <c r="BA3" t="s">
+        <v>65</v>
+      </c>
+      <c r="BB3" t="s">
         <v>93</v>
       </c>
-      <c r="AZ3">
-        <v>1</v>
-      </c>
-      <c r="BA3" t="s">
-        <v>62</v>
-      </c>
-      <c r="BB3" t="s">
-        <v>63</v>
-      </c>
-      <c r="BC3" t="s">
-        <v>64</v>
-      </c>
-      <c r="BD3">
-        <v>0</v>
-      </c>
-      <c r="BE3">
-        <v>1</v>
-      </c>
-      <c r="BF3" t="s">
-        <v>62</v>
-      </c>
-      <c r="BG3" t="s">
-        <v>65</v>
-      </c>
-      <c r="BH3" t="s">
-        <v>64</v>
-      </c>
-      <c r="BI3">
+      <c r="BC3">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{6B4B139F-5BD3-0642-96FD-B1E293BB7330}"/>
-    <hyperlink ref="AL2" r:id="rId2" xr:uid="{CD755D91-AB99-E442-AEBE-30FEAB99775E}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:BD3" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>